<commit_message>
feat: sentinal_ihsan anlatim sesi Charon-fisilti -> Algieba sakin (Ihsan geri bildirimi)
- Ihsan (P1 izleyince): 'whispering creepy olmus, sessiz olsun ama fisildamasin,
  urkutucu ve irite edici' -> fisilti talimati kaldirildi; sakin/normal ses,
  do-not-whisper acik talimat; Algieba = influencer persona sesiyle ayni (tek marka sesi)
- night-archive P1: YT'ye yerel telafi yuklemesi yapildi (yeni sesle, crf28 15MB),
  platforms_ok += youtube; yarin P2'den itibaren tum bolumler yeni sesle

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/series_data/night-archive/series_log.xlsx
+++ b/series_data/night-archive/series_log.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -830,6 +830,120 @@
       <c r="M7" t="inlineStr">
         <is>
           <t>/home/runner/work/youtube-automation/youtube-automation/output/series/night-archive/episodes/ep01/shots/shot_06.mp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:51</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>1080p</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>126.0</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>0.63</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>https://tempfile.aiquickdraw.com/v/85b58e0354063aba40d3c34701349172_1783111723.mp4</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>C:\Users\ihsan\Desktop\Antigravity\Projects\Youtube\output\series\night-archive\episodes\ep01\shots\shot_05.mp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:53</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Ihsan</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>1080p</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>105.0</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>0.525</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>https://tempfile.aiquickdraw.com/v/b94f14ac5f8ac6e9c95841103b82b93a_1783112002.mp4</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>C:\Users\ihsan\Desktop\Antigravity\Projects\Youtube\output\series\night-archive\episodes\ep01\shots\shot_06.mp4</t>
         </is>
       </c>
     </row>

</xml_diff>